<commit_message>
added online option in the book couloumn data validation.
</commit_message>
<xml_diff>
--- a/אנגלי.xlsx
+++ b/אנגלי.xlsx
@@ -5,20 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dvir\תחקור פסיכומטרי\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dvir\psychometricInvestigationWithGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B11B2A-7E2A-44C6-8FAD-4B16A4838FFF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF4A5F0-B762-4F15-866F-D27CF512F721}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="דוגמית לטאב" sheetId="5" r:id="rId1"/>
-    <sheet name="השלמת משפטים" sheetId="12" r:id="rId2"/>
+    <sheet name="דוגמית לטאב" sheetId="14" r:id="rId1"/>
+    <sheet name="השלמת משפטים" sheetId="13" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'דוגמית לטאב'!$B$2:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'השלמת משפטים'!$B$2:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'דוגמית לטאב'!$B$2:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'השלמת משפטים'!$B$2:$G$2</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>למה טעיתי</t>
   </si>
@@ -41,10 +41,13 @@
     <t>איך אשתפר</t>
   </si>
   <si>
-    <t>ספר הטעות</t>
-  </si>
-  <si>
     <t>עמוד ושאלת הטעות</t>
+  </si>
+  <si>
+    <t>הפלוס במה שעשיתי</t>
+  </si>
+  <si>
+    <t>מיקום כללי של הטעות</t>
   </si>
 </sst>
 </file>
@@ -376,42 +379,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4AEE827-035F-48C6-B2F2-CF9271AF7B67}">
-  <dimension ref="B2:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ED8C040-4361-40D2-A54B-6ECBA7350B4B}">
+  <dimension ref="B2:G2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="20.69921875" customWidth="1"/>
-    <col min="4" max="4" width="40.69921875" customWidth="1"/>
-    <col min="5" max="5" width="20.69921875" customWidth="1"/>
-    <col min="6" max="6" width="40.69921875" customWidth="1"/>
+    <col min="2" max="2" width="40.69921875" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" customWidth="1"/>
+    <col min="4" max="4" width="17.69921875" customWidth="1"/>
+    <col min="5" max="5" width="40.69921875" customWidth="1"/>
+    <col min="6" max="6" width="17.69921875" customWidth="1"/>
+    <col min="7" max="7" width="40.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:F2" xr:uid="{9143E0B2-37ED-40BA-BF74-A880F10CB732}"/>
+  <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
   <dataConsolidate/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{EE27D4B7-642F-434F-A73B-A32F69E4DB31}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1 F3:F1048576" xr:uid="{DBECB60C-6B8F-4EC4-BC7D-BFDD3056BA1F}">
       <formula1>"ידע, הבנה, כאפה"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{AAB13882-3EFF-4A7C-80C9-A055A70B9A48}">
-      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{353B4500-C815-4C3A-9200-434D4A2DAC3C}">
+      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -420,41 +428,46 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013BD43D-6B90-4D2B-838C-F64CA912F963}">
-  <dimension ref="B2:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811A6494-9384-4226-8C0A-A88B755A0B55}">
+  <dimension ref="B2:G2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="20.69921875" customWidth="1"/>
-    <col min="4" max="4" width="40.69921875" customWidth="1"/>
-    <col min="5" max="5" width="20.69921875" customWidth="1"/>
-    <col min="6" max="6" width="40.69921875" customWidth="1"/>
+    <col min="2" max="2" width="40.69921875" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" customWidth="1"/>
+    <col min="4" max="4" width="17.69921875" customWidth="1"/>
+    <col min="5" max="5" width="40.69921875" customWidth="1"/>
+    <col min="6" max="6" width="17.69921875" customWidth="1"/>
+    <col min="7" max="7" width="40.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:F2" xr:uid="{9143E0B2-37ED-40BA-BF74-A880F10CB732}"/>
+  <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
   <dataConsolidate/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{24CE509D-0918-4110-A046-184F1C580D79}">
-      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{0D4A0C2B-1B6D-4351-A2BD-738D46394707}">
+      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{ED0F5CE6-4D97-4325-A06F-FCAE311EE9D2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1 F3:F1048576" xr:uid="{951182A0-7CE2-4ED3-BA5A-FF7B2994B1B4}">
       <formula1>"ידע, הבנה, כאפה"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
added wrap text and updated data validation for every tab in any of the three file.
</commit_message>
<xml_diff>
--- a/אנגלי.xlsx
+++ b/אנגלי.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dvir\psychometricInvestigationWithGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF4A5F0-B762-4F15-866F-D27CF512F721}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146A7072-D20E-4521-80CD-70887449B9E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="דוגמית לטאב" sheetId="14" r:id="rId1"/>
-    <sheet name="השלמת משפטים" sheetId="13" r:id="rId2"/>
+    <sheet name="השלמת משפטים" sheetId="15" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'דוגמית לטאב'!$B$2:$G$2</definedName>
@@ -97,9 +97,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,17 +383,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ED8C040-4361-40D2-A54B-6ECBA7350B4B}">
-  <dimension ref="B2:G2"/>
+  <dimension ref="B1:G3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="40.69921875" customWidth="1"/>
-    <col min="3" max="3" width="18.69921875" customWidth="1"/>
-    <col min="4" max="4" width="17.69921875" customWidth="1"/>
-    <col min="5" max="5" width="40.69921875" customWidth="1"/>
-    <col min="6" max="6" width="17.69921875" customWidth="1"/>
-    <col min="7" max="7" width="40.69921875" customWidth="1"/>
+    <col min="2" max="2" width="40.69921875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.69921875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="40.69921875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.69921875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.69921875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+    </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>4</v>
@@ -410,16 +421,24 @@
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
   <dataConsolidate/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1 F3:F1048576" xr:uid="{DBECB60C-6B8F-4EC4-BC7D-BFDD3056BA1F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{DBECB60C-6B8F-4EC4-BC7D-BFDD3056BA1F}">
       <formula1>"ידע, הבנה, כאפה"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{353B4500-C815-4C3A-9200-434D4A2DAC3C}">
-      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" xr:uid="{353B4500-C815-4C3A-9200-434D4A2DAC3C}">
+      <formula1>"ספר חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -428,18 +447,26 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811A6494-9384-4226-8C0A-A88B755A0B55}">
-  <dimension ref="B2:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFEE72B-F83C-43B5-961A-ADEB3BD0B165}">
+  <dimension ref="B1:G3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="40.69921875" customWidth="1"/>
-    <col min="3" max="3" width="18.69921875" customWidth="1"/>
-    <col min="4" max="4" width="17.69921875" customWidth="1"/>
-    <col min="5" max="5" width="40.69921875" customWidth="1"/>
-    <col min="6" max="6" width="17.69921875" customWidth="1"/>
-    <col min="7" max="7" width="40.69921875" customWidth="1"/>
+    <col min="2" max="2" width="40.69921875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.69921875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="40.69921875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.69921875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.69921875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+    </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>4</v>
@@ -459,15 +486,23 @@
       <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:G2" xr:uid="{87CB5822-66D4-452B-A3EB-3E11EDA85BE8}"/>
   <dataConsolidate/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{0D4A0C2B-1B6D-4351-A2BD-738D46394707}">
-      <formula1>"חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" xr:uid="{DA950A9B-C734-4EF9-89BF-D91866D96125}">
+      <formula1>"ספר חשיבה פסיכומטרית, ספר האנגלית, גל 1, גל 2, גל 3, בחנים חמים מהתנור, סימולציה 1, סימולציה 2, סימולציה 3, סימולציה 4, סימולציה 5, סימולציה 6, סימולציה 7, סימולציה 8, סימולציה 9"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1 F3:F1048576" xr:uid="{951182A0-7CE2-4ED3-BA5A-FF7B2994B1B4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576" xr:uid="{9E998A27-FB9C-4D8D-A687-B8F59A7B1C4C}">
       <formula1>"ידע, הבנה, כאפה"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>